<commit_message>
vault backup: 2026-09-23 09:01:17
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/06_확인필요/확인필요_20260922_2216.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/06_확인필요/확인필요_20260922_2216.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AP\Documents\mynotes\01-Projects\에이팜건강-주간자금계획-자동화\자금계획_자동화\06_확인필요\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20B6C0F3-9D00-40FD-B77F-FA534A24C19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40F12D9-BE1C-4C39-A77C-533245CF18E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="안내" sheetId="1" r:id="rId1"/>
@@ -419,6 +419,9 @@
     <t>네이버 — 미집행: 당일 실제 출금에서 일치 항목 없음. 오늘 나갈 예정이면 '지출 예정(유지)', 안 나갈 것이면 '보류(제외)'를 처리 열에서 고르세요</t>
   </si>
   <si>
+    <t>지출 예정(유지)</t>
+  </si>
+  <si>
     <t>경영-20260918-015</t>
   </si>
   <si>
@@ -729,9 +732,6 @@
   </si>
   <si>
     <t>코웨이멤버쉽</t>
-  </si>
-  <si>
-    <t>보류(제외)</t>
   </si>
   <si>
     <t>예</t>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="H33" s="16"/>
       <c r="I33" s="19" t="s">
-        <v>234</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -2901,25 +2901,25 @@
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E34" s="18">
         <v>46287</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G34" s="17">
         <v>20000000</v>
       </c>
       <c r="H34" s="16"/>
       <c r="I34" s="19" t="s">
-        <v>234</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>
@@ -2928,16 +2928,16 @@
         <v>46288</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G35" s="17">
         <v>7641812</v>
       </c>
       <c r="H35" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J35" t="s">
         <v>39</v>
@@ -2945,7 +2945,7 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B36" s="16"/>
       <c r="C36" s="16"/>
@@ -2954,16 +2954,16 @@
         <v>46288</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G36" s="17">
         <v>173250</v>
       </c>
       <c r="H36" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J36" t="s">
         <v>41</v>
@@ -2971,7 +2971,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
@@ -2980,16 +2980,16 @@
         <v>46293</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G37" s="17">
         <v>2000000</v>
       </c>
       <c r="H37" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J37" t="s">
         <v>42</v>
@@ -2997,7 +2997,7 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
@@ -3006,16 +3006,16 @@
         <v>46293</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G38" s="17">
         <v>1650000</v>
       </c>
       <c r="H38" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J38" t="s">
         <v>43</v>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="16"/>
@@ -3032,16 +3032,16 @@
         <v>46293</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G39" s="17">
         <v>449429</v>
       </c>
       <c r="H39" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J39" t="s">
         <v>44</v>
@@ -3049,7 +3049,7 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B40" s="16"/>
       <c r="C40" s="16"/>
@@ -3058,16 +3058,16 @@
         <v>46294</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G40" s="17">
         <v>1348600</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J40" t="s">
         <v>46</v>
@@ -3075,7 +3075,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
@@ -3084,16 +3084,16 @@
         <v>46294</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G41" s="17">
         <v>1045000</v>
       </c>
       <c r="H41" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J41" t="s">
         <v>47</v>
@@ -3101,7 +3101,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="16"/>
@@ -3110,16 +3110,16 @@
         <v>46295</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G42" s="17">
         <v>65040941</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J42" t="s">
         <v>49</v>
@@ -3127,7 +3127,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B43" s="16"/>
       <c r="C43" s="16"/>
@@ -3136,16 +3136,16 @@
         <v>46295</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G43" s="17">
         <v>10790260</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J43" t="s">
         <v>50</v>
@@ -3153,7 +3153,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B44" s="16"/>
       <c r="C44" s="16"/>
@@ -3162,16 +3162,16 @@
         <v>46295</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G44" s="17">
         <v>8156420</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J44" t="s">
         <v>51</v>
@@ -3179,7 +3179,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
@@ -3188,16 +3188,16 @@
         <v>46295</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G45" s="17">
         <v>214586</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J45" t="s">
         <v>52</v>
@@ -3205,7 +3205,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
@@ -3214,16 +3214,16 @@
         <v>46296</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G46" s="17">
         <v>2952747</v>
       </c>
       <c r="H46" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J46" t="s">
         <v>53</v>
@@ -3266,7 +3266,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -3279,20 +3279,20 @@
     </row>
     <row r="2" spans="1:16" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="J4" s="21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L4" s="23" t="str">
         <f>IF($K$4="변경 안 함","","← 전체 일괄이 켜져 있어 아래 개별·분류별 선택은 무시됩니다. 지난 선택으로 되돌리려면 '변경 안 함'을 고르세요")</f>
@@ -3307,40 +3307,40 @@
         <v>26</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>28</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="24" x14ac:dyDescent="0.3">
@@ -3351,7 +3351,7 @@
         <v>49</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D6" s="24">
         <v>7</v>
@@ -3369,26 +3369,26 @@
         <v>81931610</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J6" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K6" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C6,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C6,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C6,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N6" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P6" s="25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="24" x14ac:dyDescent="0.3">
@@ -3396,10 +3396,10 @@
         <v>111</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D7" s="24">
         <v>4</v>
@@ -3417,17 +3417,17 @@
         <v>107542010</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J7" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K7" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C7,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C7,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C7,$M$6:$M$24,0))),"제외")))</f>
         <v>제외</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="N7" s="19" t="s">
         <v>33</v>
@@ -3436,7 +3436,7 @@
         <v>33</v>
       </c>
       <c r="P7" s="25" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="24" x14ac:dyDescent="0.3">
@@ -3447,7 +3447,7 @@
         <v>59</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D8" s="24">
         <v>6</v>
@@ -3465,26 +3465,26 @@
         <v>42006200</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K8" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C8,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C8,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C8,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N8" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P8" s="25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
@@ -3492,10 +3492,10 @@
         <v>96</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D9" s="24">
         <v>4</v>
@@ -3513,17 +3513,17 @@
         <v>55000000</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K9" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C9,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C9,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C9,$M$6:$M$24,0))),"제외")))</f>
         <v>제외</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="N9" s="19" t="s">
         <v>33</v>
@@ -3532,7 +3532,7 @@
         <v>33</v>
       </c>
       <c r="P9" s="25" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
@@ -3543,7 +3543,7 @@
         <v>76</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D10" s="24">
         <v>7</v>
@@ -3561,26 +3561,26 @@
         <v>49109500</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K10" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C10,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C10,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C10,$M$6:$M$24,0))),"비정기")))</f>
         <v>비정기</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N10" s="19" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="O10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="P10" s="25" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
@@ -3591,7 +3591,7 @@
         <v>54</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D11" s="24">
         <v>6</v>
@@ -3609,23 +3609,23 @@
         <v>30000000</v>
       </c>
       <c r="I11" s="16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J11" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K11" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C11,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C11,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C11,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N11" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -3633,10 +3633,10 @@
         <v>111</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D12" s="24">
         <v>4</v>
@@ -3654,23 +3654,23 @@
         <v>40000000</v>
       </c>
       <c r="I12" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J12" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K12" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C12,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C12,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C12,$M$6:$M$24,0))),"제외")))</f>
         <v>제외</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N12" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
@@ -3681,7 +3681,7 @@
         <v>38</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D13" s="24">
         <v>5</v>
@@ -3699,23 +3699,23 @@
         <v>29671488</v>
       </c>
       <c r="I13" s="16" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K13" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C13,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C13,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C13,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N13" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
@@ -3726,7 +3726,7 @@
         <v>60</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D14" s="24">
         <v>6</v>
@@ -3744,23 +3744,23 @@
         <v>38595390</v>
       </c>
       <c r="I14" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J14" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K14" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C14,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C14,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C14,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="N14" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
@@ -3771,7 +3771,7 @@
         <v>62</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D15" s="24">
         <v>6</v>
@@ -3789,23 +3789,23 @@
         <v>21278390</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K15" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C15,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C15,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C15,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="N15" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
@@ -3816,7 +3816,7 @@
         <v>61</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D16" s="24">
         <v>6</v>
@@ -3834,23 +3834,23 @@
         <v>22391600</v>
       </c>
       <c r="I16" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J16" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K16" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C16,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C16,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C16,$M$6:$M$24,0))),"제외")))</f>
         <v>제외</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N16" s="19" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="O16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
@@ -3861,7 +3861,7 @@
         <v>50</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D17" s="24">
         <v>6</v>
@@ -3879,23 +3879,23 @@
         <v>11946900</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K17" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C17,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C17,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C17,$M$6:$M$24,0))),"비정기")))</f>
         <v>비정기</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N17" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
@@ -3906,7 +3906,7 @@
         <v>63</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D18" s="24">
         <v>4</v>
@@ -3924,17 +3924,17 @@
         <v>11000000</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J18" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K18" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C18,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C18,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C18,$M$6:$M$24,0))),"제외")))</f>
         <v>제외</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="N18" s="19" t="s">
         <v>33</v>
@@ -3951,7 +3951,7 @@
         <v>58</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D19" s="24">
         <v>6</v>
@@ -3969,17 +3969,17 @@
         <v>9029190</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J19" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K19" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C19,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C19,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C19,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N19" s="19" t="s">
         <v>33</v>
@@ -3996,7 +3996,7 @@
         <v>51</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D20" s="24">
         <v>4</v>
@@ -4014,34 +4014,34 @@
         <v>13325600</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J20" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K20" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C20,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C20,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C20,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N20" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O20" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B21" s="16" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D21" s="24">
         <v>7</v>
@@ -4059,23 +4059,23 @@
         <v>13491445</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J21" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K21" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C21,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C21,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C21,$M$6:$M$24,0))),"비정기")))</f>
         <v>비정기</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N21" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
@@ -4086,7 +4086,7 @@
         <v>39</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D22" s="24">
         <v>6</v>
@@ -4104,23 +4104,23 @@
         <v>7789380</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J22" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C22,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C22,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C22,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N22" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
@@ -4128,10 +4128,10 @@
         <v>111</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D23" s="24">
         <v>7</v>
@@ -4149,34 +4149,34 @@
         <v>10472000</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J23" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K23" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C23,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C23,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C23,$M$6:$M$24,0))),"비정기")))</f>
         <v>비정기</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N23" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>40</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D24" s="24">
         <v>6</v>
@@ -4194,23 +4194,23 @@
         <v>10777166</v>
       </c>
       <c r="I24" s="16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J24" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K24" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C24,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C24,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C24,$M$6:$M$24,0))),"정기")))</f>
         <v>정기</v>
       </c>
       <c r="M24" s="16" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N24" s="19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -4221,7 +4221,7 @@
         <v>72</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D25" s="24">
         <v>6</v>
@@ -4239,10 +4239,10 @@
         <v>5001750</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K25" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C25,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C25,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C25,$M$6:$M$24,0))),"정기")))</f>
@@ -4257,7 +4257,7 @@
         <v>55</v>
       </c>
       <c r="C26" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D26" s="24">
         <v>6</v>
@@ -4275,10 +4275,10 @@
         <v>4494000</v>
       </c>
       <c r="I26" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K26" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C26,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C26,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C26,$M$6:$M$24,0))),"정기")))</f>
@@ -4290,10 +4290,10 @@
         <v>111</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D27" s="24">
         <v>7</v>
@@ -4311,10 +4311,10 @@
         <v>6000000</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J27" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K27" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C27,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C27,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C27,$M$6:$M$24,0))),"제외")))</f>
@@ -4329,7 +4329,7 @@
         <v>56</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D28" s="24">
         <v>5</v>
@@ -4347,10 +4347,10 @@
         <v>3003000</v>
       </c>
       <c r="I28" s="16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J28" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K28" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C28,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C28,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C28,$M$6:$M$24,0))),"정기")))</f>
@@ -4365,7 +4365,7 @@
         <v>53</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D29" s="24">
         <v>6</v>
@@ -4383,10 +4383,10 @@
         <v>3688630</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J29" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K29" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C29,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C29,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C29,$M$6:$M$24,0))),"제외")))</f>
@@ -4401,7 +4401,7 @@
         <v>66</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D30" s="24">
         <v>6</v>
@@ -4419,10 +4419,10 @@
         <v>5539200</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J30" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K30" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C30,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C30,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C30,$M$6:$M$24,0))),"제외")))</f>
@@ -4434,10 +4434,10 @@
         <v>111</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D31" s="24">
         <v>7</v>
@@ -4455,10 +4455,10 @@
         <v>3215678</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J31" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K31" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C31,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C31,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C31,$M$6:$M$24,0))),"제외")))</f>
@@ -4470,10 +4470,10 @@
         <v>111</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D32" s="24">
         <v>4</v>
@@ -4491,10 +4491,10 @@
         <v>4836318</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J32" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K32" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C32,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C32,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C32,$M$6:$M$24,0))),"제외")))</f>
@@ -4509,7 +4509,7 @@
         <v>42</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D33" s="24">
         <v>4</v>
@@ -4527,10 +4527,10 @@
         <v>2000000</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J33" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K33" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C33,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C33,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C33,$M$6:$M$24,0))),"제외")))</f>
@@ -4542,10 +4542,10 @@
         <v>111</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D34" s="24">
         <v>4</v>
@@ -4563,10 +4563,10 @@
         <v>1836000</v>
       </c>
       <c r="I34" s="16" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J34" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K34" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C34,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C34,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C34,$M$6:$M$24,0))),"비정기")))</f>
@@ -4581,7 +4581,7 @@
         <v>43</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D35" s="24">
         <v>5</v>
@@ -4599,10 +4599,10 @@
         <v>1650000</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J35" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K35" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C35,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C35,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C35,$M$6:$M$24,0))),"비정기")))</f>
@@ -4614,10 +4614,10 @@
         <v>111</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D36" s="24">
         <v>4</v>
@@ -4635,10 +4635,10 @@
         <v>5350000</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J36" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K36" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C36,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C36,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C36,$M$6:$M$24,0))),"비정기")))</f>
@@ -4653,7 +4653,7 @@
         <v>31</v>
       </c>
       <c r="C37" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D37" s="24">
         <v>4</v>
@@ -4671,10 +4671,10 @@
         <v>2200000</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J37" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K37" s="16" t="str">
         <f t="shared" ref="K37:K42" si="0">IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C37,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C37,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C37,$M$6:$M$24,0))),"제외")))</f>
@@ -4686,10 +4686,10 @@
         <v>111</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D38" s="24">
         <v>6</v>
@@ -4707,10 +4707,10 @@
         <v>2841698</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J38" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K38" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4725,7 +4725,7 @@
         <v>46</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D39" s="24">
         <v>5</v>
@@ -4743,10 +4743,10 @@
         <v>4818000</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J39" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K39" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4761,7 +4761,7 @@
         <v>47</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D40" s="24">
         <v>4</v>
@@ -4779,10 +4779,10 @@
         <v>1320000</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J40" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K40" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4797,7 +4797,7 @@
         <v>68</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D41" s="24">
         <v>6</v>
@@ -4815,10 +4815,10 @@
         <v>1650000</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J41" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K41" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4830,10 +4830,10 @@
         <v>111</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D42" s="24">
         <v>7</v>
@@ -4851,10 +4851,10 @@
         <v>1060000</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J42" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K42" s="16" t="str">
         <f t="shared" si="0"/>
@@ -4869,7 +4869,7 @@
         <v>48</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D43" s="24">
         <v>4</v>
@@ -4887,10 +4887,10 @@
         <v>908980</v>
       </c>
       <c r="I43" s="16" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J43" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K43" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C43,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C43,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C43,$M$6:$M$24,0))),"비정기")))</f>
@@ -4905,7 +4905,7 @@
         <v>44</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D44" s="24">
         <v>7</v>
@@ -4923,10 +4923,10 @@
         <v>1100000</v>
       </c>
       <c r="I44" s="16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J44" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K44" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C44,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C44,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C44,$M$6:$M$24,0))),"제외")))</f>
@@ -4941,7 +4941,7 @@
         <v>36</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D45" s="24">
         <v>6</v>
@@ -4959,10 +4959,10 @@
         <v>381700</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J45" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K45" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C45,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C45,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C45,$M$6:$M$24,0))),"제외")))</f>
@@ -4977,7 +4977,7 @@
         <v>34</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D46" s="24">
         <v>6</v>
@@ -4995,10 +4995,10 @@
         <v>227899</v>
       </c>
       <c r="I46" s="16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J46" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K46" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C46,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C46,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C46,$M$6:$M$24,0))),"정기")))</f>
@@ -5013,7 +5013,7 @@
         <v>69</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D47" s="24">
         <v>5</v>
@@ -5031,10 +5031,10 @@
         <v>220000</v>
       </c>
       <c r="I47" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J47" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K47" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C47,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C47,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C47,$M$6:$M$24,0))),"제외")))</f>
@@ -5049,7 +5049,7 @@
         <v>52</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D48" s="24">
         <v>5</v>
@@ -5067,10 +5067,10 @@
         <v>328130</v>
       </c>
       <c r="I48" s="16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J48" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K48" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C48,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C48,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C48,$M$6:$M$24,0))),"비정기")))</f>
@@ -5085,7 +5085,7 @@
         <v>70</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D49" s="24">
         <v>6</v>
@@ -5103,10 +5103,10 @@
         <v>198000</v>
       </c>
       <c r="I49" s="16" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J49" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K49" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C49,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C49,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C49,$M$6:$M$24,0))),"제외")))</f>
@@ -5121,7 +5121,7 @@
         <v>41</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D50" s="24">
         <v>4</v>
@@ -5139,10 +5139,10 @@
         <v>231000</v>
       </c>
       <c r="I50" s="16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J50" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K50" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C50,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C50,$M$6:$M$24,0)),"비정기",INDEX($N$6:$N$24,MATCH($C50,$M$6:$M$24,0))),"비정기")))</f>
@@ -5157,7 +5157,7 @@
         <v>73</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D51" s="24">
         <v>5</v>
@@ -5175,10 +5175,10 @@
         <v>253800</v>
       </c>
       <c r="I51" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J51" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K51" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C51,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C51,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C51,$M$6:$M$24,0))),"정기")))</f>
@@ -5190,10 +5190,10 @@
         <v>111</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D52" s="24">
         <v>6</v>
@@ -5211,10 +5211,10 @@
         <v>129610</v>
       </c>
       <c r="I52" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J52" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K52" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C52,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C52,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C52,$M$6:$M$24,0))),"제외")))</f>
@@ -5229,7 +5229,7 @@
         <v>45</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D53" s="24">
         <v>6</v>
@@ -5247,10 +5247,10 @@
         <v>145540</v>
       </c>
       <c r="I53" s="16" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J53" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K53" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C53,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C53,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C53,$M$6:$M$24,0))),"정기")))</f>
@@ -5265,7 +5265,7 @@
         <v>71</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D54" s="24">
         <v>4</v>
@@ -5283,10 +5283,10 @@
         <v>289440</v>
       </c>
       <c r="I54" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J54" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K54" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C54,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C54,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C54,$M$6:$M$24,0))),"제외")))</f>
@@ -5298,10 +5298,10 @@
         <v>111</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D55" s="24">
         <v>7</v>
@@ -5319,10 +5319,10 @@
         <v>100000</v>
       </c>
       <c r="I55" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J55" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K55" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C55,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C55,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C55,$M$6:$M$24,0))),"제외")))</f>
@@ -5337,7 +5337,7 @@
         <v>57</v>
       </c>
       <c r="C56" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D56" s="24">
         <v>6</v>
@@ -5355,10 +5355,10 @@
         <v>100000</v>
       </c>
       <c r="I56" s="16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J56" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K56" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C56,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C56,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C56,$M$6:$M$24,0))),"제외")))</f>
@@ -5370,10 +5370,10 @@
         <v>111</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D57" s="24">
         <v>6</v>
@@ -5391,10 +5391,10 @@
         <v>67100</v>
       </c>
       <c r="I57" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J57" s="16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K57" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C57,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C57,$M$6:$M$24,0)),"제외",INDEX($N$6:$N$24,MATCH($C57,$M$6:$M$24,0))),"제외")))</f>
@@ -5409,7 +5409,7 @@
         <v>74</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D58" s="24">
         <v>7</v>
@@ -5427,10 +5427,10 @@
         <v>33990</v>
       </c>
       <c r="I58" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J58" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K58" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C58,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C58,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C58,$M$6:$M$24,0))),"정기")))</f>
@@ -5445,7 +5445,7 @@
         <v>75</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D59" s="24">
         <v>7</v>
@@ -5463,10 +5463,10 @@
         <v>11000</v>
       </c>
       <c r="I59" s="16" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J59" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K59" s="16" t="str">
         <f>IF($K$4="전체 정기","정기",IF($K$4="전체 비정기","비정기",IFERROR(IF(INDEX($N$6:$N$24,MATCH($C59,$M$6:$M$24,0))=INDEX($O$6:$O$24,MATCH($C59,$M$6:$M$24,0)),"정기",INDEX($N$6:$N$24,MATCH($C59,$M$6:$M$24,0))),"정기")))</f>

</xml_diff>